<commit_message>
refactor: quality wolf 改名 wolf_hunt，避免跟角色 id wolf 共用 <npcId>.xxx 命名空間
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/xls/story.xlsx
+++ b/xls/story.xlsx
@@ -73,7 +73,7 @@
     <t>討伐令的殺盜賊計數器（count 開、stop 停）</t>
   </si>
   <si>
-    <t>wolf</t>
+    <t>wolf_hunt</t>
   </si>
   <si>
     <t>屠夫的生意經</t>
@@ -82,7 +82,7 @@
     <t>xi 的狼皮委託：1 殺 3 隻狼 / 2 剝狼皮 / 3 狼皮交給 karen / 4 回報 xi / 10 完成</t>
   </si>
   <si>
-    <t>wolf.kills</t>
+    <t>wolf_hunt.kills</t>
   </si>
   <si>
     <t>狼患的殺狼計數器（count 開、stop 停）</t>
@@ -361,7 +361,7 @@
     <t>黑森林的野狼氾濫，xi 的肉舖快沒貨了，想找人幫忙獵狼取皮，順便帶個口信給城裡的商人 karen。</t>
   </si>
   <si>
-    <t>前往黑森林狩獵，擊殺野狼 ({wolf.kills}/3)</t>
+    <t>前往黑森林狩獵，擊殺野狼 ({wolf_hunt.kills}/3)</t>
   </si>
   <si>
     <t>金幣 x120、斧頭 x1</t>
@@ -385,7 +385,7 @@
     <t>wolf_ask</t>
   </si>
   <si>
-    <t>wolf==0</t>
+    <t>wolf_hunt==0</t>
   </si>
   <si>
     <t>@n_wolf_ask</t>
@@ -394,26 +394,26 @@
     <t>wolf_kill</t>
   </si>
   <si>
-    <t>wolf==1 &amp;&amp; wolf.kills&gt;=3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wolf=2 ;
-stop wolf.kills</t>
+    <t>wolf_hunt==1 &amp;&amp; wolf_hunt.kills&gt;=3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wolf_hunt=2 ;
+stop wolf_hunt.kills</t>
   </si>
   <si>
     <t>wolf_pelt</t>
   </si>
   <si>
-    <t>wolf==2 &amp;&amp; item:plet:1</t>
-  </si>
-  <si>
-    <t>wolf=3</t>
+    <t>wolf_hunt==2 &amp;&amp; item:plet:1</t>
+  </si>
+  <si>
+    <t>wolf_hunt=3</t>
   </si>
   <si>
     <t>wolf_karen</t>
   </si>
   <si>
-    <t>wolf==3 &amp;&amp; item:plet:1</t>
+    <t>wolf_hunt==3 &amp;&amp; item:plet:1</t>
   </si>
   <si>
     <t>關於黑森林的狼皮</t>
@@ -425,7 +425,7 @@
     <t>wolf_report</t>
   </si>
   <si>
-    <t>wolf&gt;=1 &amp;&amp; wolf&lt;9</t>
+    <t>wolf_hunt&gt;=1 &amp;&amp; wolf_hunt&lt;9</t>
   </si>
   <si>
     <t>@n_wolf_report</t>
@@ -434,7 +434,7 @@
     <t>wolf_sell</t>
   </si>
   <si>
-    <t>wolf==2</t>
+    <t>wolf_hunt==2</t>
   </si>
   <si>
     <t>把狼皮直接賣給你</t>
@@ -447,7 +447,7 @@
   </si>
   <si>
     <t xml:space="preserve">take plet 1 ;
-wolf=9 ;
+wolf_hunt=9 ;
 gold+80</t>
   </si>
   <si>
@@ -457,7 +457,7 @@
     <t>see</t>
   </si>
   <si>
-    <t>wolf==9 &amp;&amp; !_grudge</t>
+    <t>wolf_hunt==9 &amp;&amp; !_grudge</t>
   </si>
   <si>
     <t>喂！你給我過來！</t>
@@ -472,30 +472,30 @@
     <t>最近黑森林的狼變多了，肉舖都要沒貨了……能幫我獵些狼皮回來嗎？</t>
   </si>
   <si>
-    <t xml:space="preserve">wolf=1 ;
-count wolf.kills kill:wolf</t>
+    <t xml:space="preserve">wolf_hunt=1 ;
+count wolf_hunt.kills kill:wolf</t>
   </si>
   <si>
     <t>n_wolf_report</t>
   </si>
   <si>
-    <t xml:space="preserve">wolf&lt;4 : 狼皮收集得如何了? ;
-wolf==4 : 都準備好了嗎？太好了! ;
-wolf==10 : 謝謝你，這是你的獎勵</t>
-  </si>
-  <si>
-    <t>wolf&lt;4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wolf=10 ;
+    <t xml:space="preserve">wolf_hunt&lt;4 : 狼皮收集得如何了? ;
+wolf_hunt==4 : 都準備好了嗎？太好了! ;
+wolf_hunt==10 : 謝謝你，這是你的獎勵</t>
+  </si>
+  <si>
+    <t>wolf_hunt&lt;4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wolf_hunt=10 ;
 gold+120 ;
 give axe_01 1</t>
   </si>
   <si>
-    <t>wolf==4</t>
-  </si>
-  <si>
-    <t>wolf==10</t>
+    <t>wolf_hunt==4</t>
+  </si>
+  <si>
+    <t>wolf_hunt==10</t>
   </si>
   <si>
     <t>n_wolf_karen</t>
@@ -508,7 +508,7 @@
   </si>
   <si>
     <t xml:space="preserve">take plet 1 ;
-wolf=4</t>
+wolf_hunt=4</t>
   </si>
   <si>
     <t>n_wolf_grudge</t>
@@ -534,7 +534,7 @@
     <t>wolves</t>
   </si>
   <si>
-    <t>wolf &amp;&amp; wolf&lt;9</t>
+    <t>wolf_hunt &amp;&amp; wolf_hunt&lt;9</t>
   </si>
   <si>
     <t>狼患進行中，m_03x05 出現 3 隻狼</t>
@@ -552,7 +552,7 @@
     <t>trade_ask</t>
   </si>
   <si>
-    <t>wolf==10 &amp;&amp; pelt_trade==0</t>
+    <t>wolf_hunt==10 &amp;&amp; pelt_trade==0</t>
   </si>
   <si>
     <t>@n_trade_ask</t>

</xml_diff>